<commit_message>
v7.3: retention R-1 (qKeepWeeks + Query-ImportJSON), ByRef fix in ValidateRequiredColumns, docs statuses yo->e, add compile_check/check_retention/add_keep_weeks tools, DATA/KEEP_WEEKS=52 in build books
</commit_message>
<xml_diff>
--- a/build/ReportMTO_starter.xlsx
+++ b/build/ReportMTO_starter.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\ReportMTO\build\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{498C3CD3-A222-42CF-82A8-5BBB80302B6B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C6E30E1F-B344-4E34-94E1-F25930FA2EA1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3915" yWindow="855" windowWidth="21600" windowHeight="11295" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Main" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="38">
   <si>
     <t>ReportMTO — панель управления</t>
   </si>
@@ -139,6 +139,9 @@
   </si>
   <si>
     <t>DEBUG</t>
+  </si>
+  <si>
+    <t>DATA/KEEP_WEEKS</t>
   </si>
 </sst>
 </file>
@@ -228,8 +231,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="tblVariable" displayName="tblVariable" ref="A1:B15">
-  <autoFilter ref="A1:B15" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="tblVariable" displayName="tblVariable" ref="A1:B16">
+  <autoFilter ref="A1:B16" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <tableColumns count="2">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Key"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Value"/>
@@ -566,7 +569,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:D15"/>
+  <dimension ref="A1:D16"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="28" customWidth="1"/>
@@ -700,6 +703,14 @@
       </c>
       <c r="B15">
         <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>37</v>
+      </c>
+      <c r="B16">
+        <v>52</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Report MTO: switch presentation to 4 slides (TZ v1.2, tasks T1-T10)
</commit_message>
<xml_diff>
--- a/build/ReportMTO_starter.xlsx
+++ b/build/ReportMTO_starter.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\ReportMTO\build\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C6E30E1F-B344-4E34-94E1-F25930FA2EA1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0B8E06B1-7E4A-4253-8397-558BC52EECD4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="39">
   <si>
     <t>ReportMTO — панель управления</t>
   </si>
@@ -142,6 +142,9 @@
   </si>
   <si>
     <t>DATA/KEEP_WEEKS</t>
+  </si>
+  <si>
+    <t>REPORT/RETENTION_WEEKS</t>
   </si>
 </sst>
 </file>
@@ -231,8 +234,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="tblVariable" displayName="tblVariable" ref="A1:B16">
-  <autoFilter ref="A1:B16" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="tblVariable" displayName="tblVariable" ref="A1:B17">
+  <autoFilter ref="A1:B17" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <tableColumns count="2">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Key"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Value"/>
@@ -569,7 +572,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:D16"/>
+  <dimension ref="A1:D17"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="28" customWidth="1"/>
@@ -711,6 +714,11 @@
       </c>
       <c r="B16">
         <v>52</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>38</v>
       </c>
     </row>
   </sheetData>

</xml_diff>